<commit_message>
adicion de carpeta con ejemplo y paso a paso para la creacion de una funcion aws lambda desde CLI
</commit_message>
<xml_diff>
--- a/session_5/ComandosBasicos_AZ_AWS_GCP.xlsx
+++ b/session_5/ComandosBasicos_AZ_AWS_GCP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\code\bsginstitute\pythonde\session_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E09ADD6-E7D1-4755-8B8C-B0E0871CC767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A436944-9BFA-44D7-9C8B-5C28B4CE0C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93105" yWindow="0" windowWidth="38610" windowHeight="20985" xr2:uid="{2F0E1C98-7F41-40C4-8A05-B485CF49C4B9}"/>
+    <workbookView xWindow="-93105" yWindow="0" windowWidth="38610" windowHeight="10545" xr2:uid="{2F0E1C98-7F41-40C4-8A05-B485CF49C4B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -421,35 +421,6 @@
   <dxfs count="9">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <color theme="0"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="medium">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -628,6 +599,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="medium">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF000000"/>
+        </top>
         <bottom style="medium">
           <color rgb="FF000000"/>
         </bottom>
@@ -635,18 +615,38 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="0"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FF000000"/>
         </left>
         <right style="medium">
           <color rgb="FF000000"/>
         </right>
-        <top style="medium">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FF000000"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -663,13 +663,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D3234EB2-24CA-40B6-A631-9C866DDEAE41}" name="Table1" displayName="Table1" ref="C4:G16" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D3234EB2-24CA-40B6-A631-9C866DDEAE41}" name="Table1" displayName="Table1" ref="C4:G16" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9F811EAE-EA55-4004-A080-47768C8ED010}" name="Categoría" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{82E1B050-7974-4154-9EEE-2002EFB12F70}" name="Operación" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{09FE7526-B02E-428E-9F4D-B606160CDCAB}" name="AWS CLI (aws)" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{4CAEAF13-A921-432E-9CE6-5BB5FFD8E148}" name="Azure CLI (az)" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{9C78E7D7-D29D-4D75-AC91-80104E372B0E}" name="Google Cloud CLI (gcloud)" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9F811EAE-EA55-4004-A080-47768C8ED010}" name="Categoría" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{82E1B050-7974-4154-9EEE-2002EFB12F70}" name="Operación" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{09FE7526-B02E-428E-9F4D-B606160CDCAB}" name="AWS CLI (aws)" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{4CAEAF13-A921-432E-9CE6-5BB5FFD8E148}" name="Azure CLI (az)" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{9C78E7D7-D29D-4D75-AC91-80104E372B0E}" name="Google Cloud CLI (gcloud)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -995,6 +995,7 @@
   <dimension ref="C4:G16"/>
   <sheetFormatPr defaultColWidth="17.6640625" defaultRowHeight="14.4"/>
   <cols>
+    <col min="3" max="3" width="18.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="50.6640625" customWidth="1"/>
     <col min="6" max="6" width="53.6640625" customWidth="1"/>

</xml_diff>